<commit_message>
A3: lộ trình 56 bài Nền phát âm và HSK 1 dựng từ đề cương; đặc tả 1.7
- Người dùng không có 贯通中文 nên bỏ đối chiếu giáo trình; giáo trình thành
  tài liệu tham khảo không bắt buộc (mục 2, 3.2, 4.3, 13).
- tools/lo-trinh/hsk1.mjs: 8 bài Nền phát âm, 48 bài HSK 1 chia 5 cụm,
  đủ 300 từ và 70 điểm ngữ pháp, mỗi bài HSK 1 có 4–8 từ.
- tools/tao-lo-trinh.mjs kiểm tra lộ trình, sinh docs/lo-trinh-hsk1.md và
  tools/mau/bai-hsk1.csv để nhập vào tab Bai; mẫu Sheet điền sẵn tab Bai.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VpJF8PVewhBZxCThUMUJ9V
</commit_message>
<xml_diff>
--- a/tools/mau/xinyu-noi-dung.xlsx
+++ b/tools/mau/xinyu-noi-dung.xlsx
@@ -108,7 +108,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tab Tu, Chu, NguPhap đã điền sẵn danh sách HSK 1 của đề cương thi 11/2025 (300 từ, 246 chữ nhận biết, 70 điểm ngữ pháp). Không đổi Mã, Mã đề cương, Từ, Cấp của các dòng này.</t>
+          <t xml:space="preserve">Tab Tu, Chu, NguPhap đã điền sẵn danh sách HSK 1 của đề cương thi 11/2025 (300 từ, 246 chữ nhận biết, 70 điểm ngữ pháp); tab Bai điền sẵn 56 bài theo docs/lo-trinh-hsk1.md. Không đổi Mã, Mã đề cương, Từ, Cấp của các dòng này.</t>
         </is>
       </c>
     </row>
@@ -1776,6 +1776,2116 @@
       <c r="R1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nền phát âm</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bốn thanh điệu</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nghe và đọc đúng bốn thanh trên âm tiết đơn</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nền phát âm</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Âm đầu (1): b p m f d t n l g k h</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Phân biệt âm bật hơi và không bật hơi</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nền phát âm</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Âm đầu (2): j q x zh ch sh r z c s</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Phân biệt ba nhóm âm dễ nhầm với tiếng Việt</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C5">
+        <v>4</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nền phát âm</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vần đơn và vần ghép</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đọc đúng vần, gồm ü và e</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C6">
+        <v>5</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nền phát âm</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vần mũi</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Phân biệt -n và -ng</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C7">
+        <v>6</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nền phát âm</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20 cặp thanh</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đọc liền hai âm tiết với 20 tổ hợp thanh</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C8">
+        <v>7</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nền phát âm</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thanh nhẹ và biến điệu</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đọc thanh nhẹ, biến điệu thanh 3, 一 và 不</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C9">
+        <v>8</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nền phát âm</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lời chào</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chào, cảm ơn, xin lỗi, tạm biệt</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">你好、谢谢、不客气、再见、对不起、没关系</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-45</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-01</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C10">
+        <v>9</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tôi là ai</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nói mình là ai bằng câu 是</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">我、你、他、她、是、人</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-09、NP1-52、NP1-35、NP1-38、NP1-42、NP1-46</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-02</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C11">
+        <v>10</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hỏi tên</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hỏi và nói tên</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">叫、什么、名字、您、请问</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-48、NP1-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-03</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C12">
+        <v>11</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Phải không?</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hỏi có/không, phủ định và hỏi lại</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">吗、不、呢、也、们、我们、你们</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-47、NP1-20、NP1-19、NP1-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-04</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C13">
+        <v>12</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quốc tịch</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hỏi và nói người nước nào</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中国、国、哪、他们、她们、都</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-16、NP1-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-05</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C14">
+        <v>13</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Học tiếng Trung</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nói mình học và biết nói tiếng gì</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">学、学习、汉语、中文、说、会1</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-06</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C15">
+        <v>14</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thầy và trò</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Giới thiệu thầy cô, bạn học</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">老师、学生、同学、大学、大学生、的</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-24、NP1-39</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-07</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C16">
+        <v>15</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Làm quen</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nói vui được làm quen</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">朋友、认识、很、好、高兴、男朋友、女朋友</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-43、NP1-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-08</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C17">
+        <v>16</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đây là ai?</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hỏi người này, người kia là ai</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">谁、这、那、这个、那个、先生、女士</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-10、NP1-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-09</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C18">
+        <v>17</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nghề nghiệp</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nói làm nghề gì, làm ở đâu</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">工作、医生、公司、做、在、男、女</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-21、NP1-31、NP1-33</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-10</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C19">
+        <v>18</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Biết chữ Hán</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nói biết, có thể làm gì</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">知道、汉字、字、写、能、可以</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-06、NP1-49</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-11</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C20">
+        <v>19</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đếm từ 1 đến 8</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đếm và đọc số nhỏ</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">一、二、三、四、五、六、七、八</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-12</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C21">
+        <v>20</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Số lớn</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đọc số đến hàng nghìn, dùng 二 và 两</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">九、十、百、千、零、两1</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-13</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C22">
+        <v>21</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gia đình tôi</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nói nhà có mấy người</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">家、家人、爸爸、妈妈、口、有</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-53、NP1-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-14</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C23">
+        <v>22</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Anh chị em</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nói có hay không có anh chị em</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">哥哥、姐姐、弟弟、妹妹、和1、没（有）</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-22、NP1-23、NP1-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-15</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C24">
+        <v>23</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tuổi</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hỏi và nói tuổi</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">岁、几、多、大、孩子、儿子、女儿</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-36</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-16</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C25">
+        <v>24</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Con vật nuôi</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đếm vật bằng lượng từ</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">狗、猫、只、个、它、它们</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-32</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-17</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C26">
+        <v>25</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ngày tháng</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hỏi và nói hôm nay ngày mấy</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">年、月、日、号、今天、明天、昨天</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-14、NP1-44、NP1-69</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-18</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C27">
+        <v>26</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thứ và năm</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nói thứ trong tuần và năm</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">星期、星期日、星期天、今年、明年、去年</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-19</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C28">
+        <v>27</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mấy giờ rồi</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hỏi và nói giờ</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">现在、点1、分、半、时候、第</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-70、NP1-68、NP1-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-20</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C29">
+        <v>28</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Các buổi trong ngày</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nói làm gì vào buổi nào</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">早上、上午、中午、下午、晚上、白天</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-40</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-21</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C30">
+        <v>29</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ăn gì?</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nói muốn ăn gì</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">吃、饭、米饭、菜、想、要</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-22</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C31">
+        <v>30</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Uống gì?</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gọi đồ uống</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">喝、茶、水、牛奶、杯子、一点儿</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-23</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C32">
+        <v>31</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Món Trung Hoa</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nói món nào ngon</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">包子、饺子、面条儿、面包、鸡蛋、好吃</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-24</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C33">
+        <v>32</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ba bữa ăn</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rủ ăn cơm, nấu cơm</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">早饭、午饭、晚饭、做饭、饭店、吧</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-26、NP1-50</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-25</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C34">
+        <v>33</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hoa quả</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nói thích gì</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">水果、苹果、喜欢、爱、些、一些</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-26</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C35">
+        <v>34</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bao nhiêu tiền?</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hỏi giá và trả tiền</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">买、卖、钱、多少、块、元</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-67</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-27</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C36">
+        <v>35</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đắt quá!</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Khen chê giá cả</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">贵、便宜、太、非常、少、了</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-63、NP1-51</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-28</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C37">
+        <v>36</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quần áo</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chọn quần áo theo cỡ</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">衣服、件、穿、漂亮、小</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-37</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-29</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C38">
+        <v>37</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đi siêu thị</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nói đã mua những gì</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">超市、商店、东西、还、本1、书</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-61、NP1-62、NP1-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-30</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C39">
+        <v>38</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cửa hàng mới</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tả cửa hàng</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">店、书店、新、真、有的、有些</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-31</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C40">
+        <v>39</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ở đâu?</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hỏi và chỉ chỗ</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">哪儿、这儿、那儿、哪里、这里、那里</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-32</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C41">
+        <v>40</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trên dưới trong ngoài</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nói đồ vật ở vị trí nào</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">上、下、里、外、前、后</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-03、NP1-34、NP1-54</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-33</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C42">
+        <v>41</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bên này, bên kia</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tả trong phòng có gì</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">边、这边、那边、外边、桌子、椅子</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-55</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-34</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C43">
+        <v>42</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nhà ở</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nói mình ở đâu, phòng có gì</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">住、房间、电脑、电视、这些、那些</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-35</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C44">
+        <v>43</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trường học</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nói học ở trường nào</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">学校、小学、中学、小学生、中学生、小朋友</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-36</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C45">
+        <v>44</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đi và về</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nói đi đâu để làm gì</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">去、来、到、回、哪个、哪些</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-56</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-37</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C46">
+        <v>45</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Phương tiện</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nói đi bằng gì</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">车、出租车、火车、飞机、坐、怎么</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-57</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-38</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C47">
+        <v>46</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đi làm, đi học</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nói giờ đi làm, đi học</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">开、开车、上学、上班、下班、对</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-39</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C48">
+        <v>47</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đi khám bệnh</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nói mình bị ốm</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">医院、病、生病、看病、有（一）点儿、再</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-40</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C49">
+        <v>48</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đi xem phim</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rủ đi xem phim</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">电影、电影院、看、看见、好看、给</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-58</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-41</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C50">
+        <v>49</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gọi điện thoại</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gọi điện hỏi có việc gì</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">打电话、电话、手机、喂1、事、没事</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-42</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C51">
+        <v>50</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hẹn gặp</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hẹn giờ và chỗ gặp</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">时间、见、忙、怎么样、一下、找</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-41</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-43</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C52">
+        <v>51</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Một ngày của tôi</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kể giờ dậy, giờ ngủ</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">起床、睡觉、睡、休息、早、晚</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-44</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C53">
+        <v>52</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đang làm gì?</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nói đang làm gì và làm bao lâu</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">正在、读、读书、小时、分钟、天</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-17、NP1-64、NP1-65、NP1-66</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-45</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C54">
+        <v>53</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thời tiết</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nói thời tiết hôm nay</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">天气、冷、热、下雨、雨、雪</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-46</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C55">
+        <v>54</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sở thích</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nói thích làm gì lúc rảnh</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">听、歌、唱、好听、玩、好玩儿</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NP1-59、NP1-60</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-47</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C56">
+        <v>55</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trong lớp học</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hỏi thầy cô khi chưa hiểu</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">课、上课、下课、说话、问、问题、听见</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H1-48</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp</t>
+        </is>
+      </c>
+      <c r="C57">
+        <v>56</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSK 1</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mời và khuyên</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mời mọi người, khuyên đừng làm gì, nói ý kiến</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">请、大家、不要、觉得、一半</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
A4: nội dung Nền phát âm, tab PhatAm và công cụ điền nội dung vào Sheet
- tools/noi-dung/a4-phat-am.mjs: 76 mục phát âm (thanh điệu, âm đầu, vần, quy tắc) cho PA01–PA07, 20 cặp thanh, 72 câu hỏi, 8 câu chào PA08, cột còn trống của bài PA01–PA08, nghĩa 53 từ ví dụ, ngữ pháp NP1-45.
- Tab PhatAm mới (phat-am.json) và cột Âm thanh cho CauHoi; kiểm tra âm tiết, chữ đọc mẫu (CC-CEDICT), âm thanh của câu hỏi nghe.
- tools/dien-noi-dung.mjs: đọc Sheet, chỉ điền ô trống và thêm dòng mới, ghi tools/ra/xinyu-noi-dung.xlsx, chạy thử kiểm tra trên các dòng vừa soạn.
- Tách đọc nguồn (lib/nguon.mjs) và dựng tab Sheet (lib/mau-sheet.mjs) để dùng chung; 3 kiểm thử mới.
- Đặc tả 1.8; cập nhật CLAUDE.md, README, mẫu Sheet, tiến độ.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M8KJhEhxZcoU6ZFcV1DuTm
</commit_message>
<xml_diff>
--- a/tools/mau/xinyu-noi-dung.xlsx
+++ b/tools/mau/xinyu-noi-dung.xlsx
@@ -9,10 +9,11 @@
     <sheet name="NguPhap" sheetId="5" r:id="rId5"/>
     <sheet name="Cau" sheetId="6" r:id="rId6"/>
     <sheet name="CauHoi" sheetId="7" r:id="rId7"/>
-    <sheet name="CapThanh" sheetId="8" r:id="rId8"/>
-    <sheet name="CapDeNham" sheetId="9" r:id="rId9"/>
-    <sheet name="Truyen" sheetId="10" r:id="rId10"/>
-    <sheet name="CanSua" sheetId="11" r:id="rId11"/>
+    <sheet name="PhatAm" sheetId="8" r:id="rId8"/>
+    <sheet name="CapThanh" sheetId="9" r:id="rId9"/>
+    <sheet name="CapDeNham" sheetId="10" r:id="rId10"/>
+    <sheet name="Truyen" sheetId="11" r:id="rId11"/>
+    <sheet name="CanSua" sheetId="12" r:id="rId12"/>
   </sheets>
 </workbook>
 </file>
@@ -1119,7 +1120,7 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Từ, chữ hoặc mã ngữ pháp mà câu hỏi kiểm tra.</t>
+          <t xml:space="preserve">Từ, chữ, mã ngữ pháp, mã phát âm (tab PhatAm) hoặc mã cặp thanh mà câu hỏi kiểm tra.</t>
         </is>
       </c>
     </row>
@@ -1138,155 +1139,155 @@
     <row r="87">
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đáp án đúng</t>
-        </is>
-      </c>
-      <c r="C87" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">có</t>
+          <t xml:space="preserve">Âm thanh</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thứ được phát ở câu hỏi nghe: một từ ở tab Tu, mã câu ở tab Cau, hoặc một âm tiết Pinyin có ở cột Âm tiết ví dụ của tab PhatAm.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đáp án sai 1</t>
+          <t xml:space="preserve">Đáp án đúng</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">có</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nhầm với 1</t>
-        </is>
-      </c>
-      <c r="D89" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vì sao người học có thể chọn đáp án sai này.</t>
+          <t xml:space="preserve">Đáp án sai 1</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đáp án sai 2</t>
+          <t xml:space="preserve">Nhầm với 1</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vì sao người học có thể chọn đáp án sai này.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nhầm với 2</t>
+          <t xml:space="preserve">Đáp án sai 2</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đáp án sai 3</t>
+          <t xml:space="preserve">Nhầm với 2</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nhầm với 3</t>
+          <t xml:space="preserve">Đáp án sai 3</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lời giải</t>
+          <t xml:space="preserve">Nhầm với 3</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="B95" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Lời giải</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="B96" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Ghi chú</t>
         </is>
       </c>
-      <c r="D95" s="2" t="inlineStr">
+      <c r="D96" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Ghi chú khi soạn, không xuất ra app.</t>
         </is>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CapThanh</t>
-        </is>
-      </c>
-      <c r="B96" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">(Cặp thanh)</t>
-        </is>
-      </c>
-    </row>
     <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PhatAm</t>
+        </is>
+      </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mã</t>
-        </is>
-      </c>
-      <c r="C97" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">có</t>
-        </is>
-      </c>
-      <c r="D97" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Mã cặp thanh, ví dụ CT11.</t>
+          <t xml:space="preserve">(Phát âm)</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trạng thái</t>
+          <t xml:space="preserve">Mã</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">có</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp hoặc đã kiểm tra. Chỉ dòng “đã kiểm tra” và không có lỗi mới được xuất ra JSON. Chọn: nháp, đã kiểm tra.</t>
+          <t xml:space="preserve">Mã mục phát âm: mã bài, gạch nối, số thứ tự, ví dụ PA02-01.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tổ hợp</t>
-        </is>
-      </c>
-      <c r="C99" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">có</t>
+          <t xml:space="preserve">Trạng thái</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Thanh của hai âm tiết, ví dụ 3-3; thanh nhẹ ghi 0, ví dụ 1-0.</t>
+          <t xml:space="preserve">nháp hoặc đã kiểm tra. Chỉ dòng “đã kiểm tra” và không có lỗi mới được xuất ra JSON. Chọn: nháp, đã kiểm tra.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cách đọc thực tế</t>
+          <t xml:space="preserve">Bài</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">có</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ví dụ 3-3 đọc thành 2-3.</t>
+          <t xml:space="preserve">Mã bài Nền phát âm. Thứ tự các mục trong bài là thứ tự dòng.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Từ ví dụ</t>
+          <t xml:space="preserve">Loại</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
@@ -1296,101 +1297,96 @@
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Từ hai âm tiết ở tab Tu.</t>
+          <t xml:space="preserve">Chọn: thanh điệu, âm đầu, vần, quy tắc.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ghi chú</t>
+          <t xml:space="preserve">Ký hiệu</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">có</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ghi chú khi soạn, không xuất ra app.</t>
+          <t xml:space="preserve">Âm đầu, vần hoặc tên thanh, quy tắc, ví dụ zh, üe, Thanh 3, Biến điệu của 不.</t>
         </is>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CapDeNham</t>
-        </is>
-      </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">(Cặp dễ nhầm)</t>
+          <t xml:space="preserve">Cách đọc</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">có</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cách đặt lưỡi, môi, hơi, cao độ; viết cho người Việt.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mã</t>
-        </is>
-      </c>
-      <c r="C104" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">có</t>
+          <t xml:space="preserve">So sánh với tiếng Việt</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mã cặp, ví dụ DN001.</t>
+          <t xml:space="preserve">Âm tiếng Việt gần nhất và chỗ khác.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trạng thái</t>
-        </is>
-      </c>
-      <c r="D105" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">nháp hoặc đã kiểm tra. Chỉ dòng “đã kiểm tra” và không có lỗi mới được xuất ra JSON. Chọn: nháp, đã kiểm tra.</t>
+          <t xml:space="preserve">Lỗi người Việt hay mắc</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Các mục</t>
-        </is>
-      </c>
-      <c r="C106" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">có</t>
+          <t xml:space="preserve">Âm tiết ví dụ</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Từ hoặc chữ dễ nhầm với nhau, ví dụ 买, 卖.</t>
+          <t xml:space="preserve">Âm tiết Pinyin có dấu thanh, mỗi mục một âm tiết, ví dụ bā, pá.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Giải thích</t>
-        </is>
-      </c>
-      <c r="C107" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">có</t>
+          <t xml:space="preserve">Chữ đọc mẫu</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mỗi âm tiết ví dụ một chữ Hán đọc đúng âm tiết đó, cùng thứ tự; chỉ dùng để tạo âm thanh, app không hiển thị.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Câu hỏi</t>
+          <t xml:space="preserve">Từ ví dụ</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mã câu hỏi phân biệt ở tab CauHoi.</t>
+          <t xml:space="preserve">Từ ở tab Tu minh họa mục này.</t>
         </is>
       </c>
     </row>
@@ -1409,12 +1405,12 @@
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Truyen</t>
+          <t xml:space="preserve">CapThanh</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">(Truyện)</t>
+          <t xml:space="preserve">(Cặp thanh)</t>
         </is>
       </c>
     </row>
@@ -1431,7 +1427,7 @@
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mã truyện, ví dụ TR001. Câu của truyện nằm ở tab Cau với cột Bài là mã truyện.</t>
+          <t xml:space="preserve">Mã cặp thanh, ví dụ CT11.</t>
         </is>
       </c>
     </row>
@@ -1450,7 +1446,7 @@
     <row r="113">
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sau bài</t>
+          <t xml:space="preserve">Tổ hợp</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
@@ -1460,108 +1456,301 @@
       </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mở sau bài này; từ đã học tính đến bài này.</t>
+          <t xml:space="preserve">Thanh của hai âm tiết, ví dụ 3-3; thanh nhẹ ghi 0, ví dụ 1-0.</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tiêu đề</t>
-        </is>
-      </c>
-      <c r="C114" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">có</t>
+          <t xml:space="preserve">Cách đọc thực tế</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ví dụ 3-3 đọc thành 2-3.</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Từ mới</t>
+          <t xml:space="preserve">Từ ví dụ</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">có</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tối đa 3 từ chưa học dùng trong truyện.</t>
+          <t xml:space="preserve">Từ hai âm tiết ở tab Tu.</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Câu hỏi</t>
+          <t xml:space="preserve">Ghi chú</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mã câu hỏi hiểu ở tab CauHoi.</t>
+          <t xml:space="preserve">Ghi chú khi soạn, không xuất ra app.</t>
         </is>
       </c>
     </row>
     <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CapDeNham</t>
+        </is>
+      </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ghi chú</t>
-        </is>
-      </c>
-      <c r="D117" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ghi chú khi soạn, không xuất ra app.</t>
+          <t xml:space="preserve">(Cặp dễ nhầm)</t>
         </is>
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CanSua</t>
-        </is>
-      </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">(Nội dung cần sửa)</t>
+          <t xml:space="preserve">Mã</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">có</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mã cặp, ví dụ DN001.</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ngày</t>
+          <t xml:space="preserve">Trạng thái</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp hoặc đã kiểm tra. Chỉ dòng “đã kiểm tra” và không có lỗi mới được xuất ra JSON. Chọn: nháp, đã kiểm tra.</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mục</t>
+          <t xml:space="preserve">Các mục</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">có</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mã từ, câu hoặc câu hỏi được báo lỗi.</t>
+          <t xml:space="preserve">Từ hoặc chữ dễ nhầm với nhau, ví dụ 买, 卖.</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nội dung</t>
-        </is>
-      </c>
-      <c r="D121" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Danh sách xuất từ app (màn 29) dán vào đây.</t>
+          <t xml:space="preserve">Giải thích</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">có</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="B122" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Câu hỏi</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mã câu hỏi phân biệt ở tab CauHoi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ghi chú</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ghi chú khi soạn, không xuất ra app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Truyen</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(Truyện)</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mã</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">có</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mã truyện, ví dụ TR001. Câu của truyện nằm ở tab Cau với cột Bài là mã truyện.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trạng thái</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nháp hoặc đã kiểm tra. Chỉ dòng “đã kiểm tra” và không có lỗi mới được xuất ra JSON. Chọn: nháp, đã kiểm tra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sau bài</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">có</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mở sau bài này; từ đã học tính đến bài này.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tiêu đề</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">có</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Từ mới</t>
+        </is>
+      </c>
+      <c r="D129" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tối đa 3 từ chưa học dùng trong truyện.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Câu hỏi</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mã câu hỏi hiểu ở tab CauHoi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ghi chú</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ghi chú khi soạn, không xuất ra app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CanSua</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(Nội dung cần sửa)</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ngày</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mục</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mã từ, câu hoặc câu hỏi được báo lỗi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nội dung</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Danh sách xuất từ app (màn 29) dán vào đây.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="B136" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Đã xử lý</t>
         </is>
       </c>
-      <c r="D122" s="2" t="inlineStr">
+      <c r="D136" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Ghi x khi đã sửa xong.</t>
         </is>
@@ -1572,6 +1761,58 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <cols>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="35" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="30" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mã</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trạng thái</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Các mục</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Giải thích</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Câu hỏi</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ghi chú</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B1000">
+      <formula1>"nháp,đã kiểm tra"</formula1>
+    </dataValidation>
+  </dataValidations>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1629,7 +1870,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -19505,15 +19746,16 @@
     <col min="5" max="5" width="8" customWidth="1"/>
     <col min="6" max="6" width="15" customWidth="1"/>
     <col min="7" max="7" width="35" customWidth="1"/>
-    <col min="8" max="8" width="15" customWidth="1"/>
+    <col min="8" max="8" width="12" customWidth="1"/>
     <col min="9" max="9" width="15" customWidth="1"/>
     <col min="10" max="10" width="15" customWidth="1"/>
     <col min="11" max="11" width="15" customWidth="1"/>
     <col min="12" max="12" width="15" customWidth="1"/>
     <col min="13" max="13" width="15" customWidth="1"/>
     <col min="14" max="14" width="15" customWidth="1"/>
-    <col min="15" max="15" width="35" customWidth="1"/>
-    <col min="16" max="16" width="30" customWidth="1"/>
+    <col min="15" max="15" width="15" customWidth="1"/>
+    <col min="16" max="16" width="35" customWidth="1"/>
+    <col min="17" max="17" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -19554,45 +19796,50 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">Âm thanh</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Đáp án đúng</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Đáp án sai 1</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Nhầm với 1</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Đáp án sai 2</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Nhầm với 2</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Đáp án sai 3</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Nhầm với 3</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Lời giải</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Ghi chú</t>
         </is>
@@ -19616,9 +19863,15 @@
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="8" customWidth="1"/>
-    <col min="4" max="4" width="25" customWidth="1"/>
-    <col min="5" max="5" width="20" customWidth="1"/>
-    <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="40" customWidth="1"/>
+    <col min="7" max="7" width="30" customWidth="1"/>
+    <col min="8" max="8" width="30" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
+    <col min="10" max="10" width="15" customWidth="1"/>
+    <col min="11" max="11" width="15" customWidth="1"/>
+    <col min="12" max="12" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -19634,29 +19887,62 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tổ hợp</t>
+          <t xml:space="preserve">Bài</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cách đọc thực tế</t>
+          <t xml:space="preserve">Loại</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">Ký hiệu</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cách đọc</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">So sánh với tiếng Việt</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lỗi người Việt hay mắc</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Âm tiết ví dụ</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chữ đọc mẫu</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Từ ví dụ</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Ghi chú</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B1000">
       <formula1>"nháp,đã kiểm tra"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D1000">
+      <formula1>"thanh điệu,âm đầu,vần,quy tắc"</formula1>
     </dataValidation>
   </dataValidations>
 </worksheet>
@@ -19667,9 +19953,9 @@
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="35" customWidth="1"/>
-    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="3" max="3" width="8" customWidth="1"/>
+    <col min="4" max="4" width="25" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
     <col min="6" max="6" width="30" customWidth="1"/>
   </cols>
   <sheetData>
@@ -19686,17 +19972,17 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Các mục</t>
+          <t xml:space="preserve">Tổ hợp</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Giải thích</t>
+          <t xml:space="preserve">Cách đọc thực tế</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Câu hỏi</t>
+          <t xml:space="preserve">Từ ví dụ</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">

</xml_diff>